<commit_message>
Docs: README event status section, US02/US03 test case sheets, coverage reports
- README: /events endpoints and who may use them; "Event status (US13)" section
  (the 8 statuses, allowed transitions, always use change_status(), who is involved);
  events now come from the backend, no sample data
- docs/testing: US03 functional test cases (13/13 pass); US02 sheet updated
  (TC-014 to re-run: attendees now see only Confirmed events)
- coverage_reports: US02, US03 and US13 runs (text reports + history.csv)
</commit_message>
<xml_diff>
--- a/docs/testing/US02_RBAC_Test_Cases.xlsx
+++ b/docs/testing/US02_RBAC_Test_Cases.xlsx
@@ -159,6 +159,9 @@
     <xf numFmtId="0" fontId="4" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="5" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="5" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
@@ -176,9 +179,6 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="10" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -635,7 +635,7 @@
       </c>
       <c r="B6" s="4" t="inlineStr">
         <is>
-          <t>Check an attendee sees only published events open for registration</t>
+          <t>Check an attendee sees only confirmed events open for registration</t>
         </is>
       </c>
       <c r="C6" s="4" t="inlineStr">
@@ -643,14 +643,14 @@
           <t>View only authorised events</t>
         </is>
       </c>
-      <c r="D6" s="5" t="inlineStr">
-        <is>
-          <t>Pass</t>
+      <c r="D6" s="7" t="inlineStr">
+        <is>
+          <t>Not Executed</t>
         </is>
       </c>
       <c r="E6" s="6" t="inlineStr">
         <is>
-          <t>NA</t>
+          <t>Rule changed 08/10/2026: attendees see only Confirmed events (an approved event's venue/date may still change). Covered by automated tests: tests/us02_rbac/event-visibility.unit.test.ts, tests/us03_us04_event_request/test_list_events.py.</t>
         </is>
       </c>
     </row>
@@ -913,7 +913,7 @@
           <t>Server-side enforcement</t>
         </is>
       </c>
-      <c r="D16" s="7" t="inlineStr">
+      <c r="D16" s="8" t="inlineStr">
         <is>
           <t>Blocked</t>
         </is>
@@ -925,56 +925,56 @@
       </c>
     </row>
     <row r="18">
-      <c r="C18" s="8" t="inlineStr">
+      <c r="C18" s="9" t="inlineStr">
         <is>
           <t>Pass</t>
         </is>
       </c>
-      <c r="D18" s="9">
+      <c r="D18" s="10">
         <f>COUNTIF($D$5:$D$16,"Pass")</f>
         <v/>
       </c>
     </row>
     <row r="19">
-      <c r="C19" s="8" t="inlineStr">
+      <c r="C19" s="9" t="inlineStr">
         <is>
           <t>Fail</t>
         </is>
       </c>
-      <c r="D19" s="9">
+      <c r="D19" s="10">
         <f>COUNTIF($D$5:$D$16,"Fail")</f>
         <v/>
       </c>
     </row>
     <row r="20">
-      <c r="C20" s="8" t="inlineStr">
+      <c r="C20" s="9" t="inlineStr">
         <is>
           <t>Not Executed</t>
         </is>
       </c>
-      <c r="D20" s="9">
+      <c r="D20" s="10">
         <f>COUNTIF($D$5:$D$16,"Not Executed")</f>
         <v/>
       </c>
     </row>
     <row r="21">
-      <c r="C21" s="8" t="inlineStr">
+      <c r="C21" s="9" t="inlineStr">
         <is>
           <t>Blocked</t>
         </is>
       </c>
-      <c r="D21" s="9">
+      <c r="D21" s="10">
         <f>COUNTIF($D$5:$D$16,"Blocked")</f>
         <v/>
       </c>
     </row>
     <row r="22">
-      <c r="C22" s="8" t="inlineStr">
+      <c r="C22" s="9" t="inlineStr">
         <is>
           <t>Total</t>
         </is>
       </c>
-      <c r="D22" s="8">
+      <c r="D22" s="9">
         <f>SUM(D18:D21)</f>
         <v/>
       </c>
@@ -1002,74 +1002,74 @@
   </cols>
   <sheetData>
     <row r="1" ht="36" customHeight="1">
-      <c r="A1" s="10" t="inlineStr">
+      <c r="A1" s="11" t="inlineStr">
         <is>
           <t>Test Case - US02 Role-Based Access Control</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="11" t="inlineStr">
+      <c r="A2" s="12" t="inlineStr">
         <is>
           <t>Blue = test case specification (written once)   Yellow = test execution record (fill in per run)</t>
         </is>
       </c>
     </row>
     <row r="4" ht="15" customHeight="1">
-      <c r="A4" s="12" t="inlineStr">
+      <c r="A4" s="13" t="inlineStr">
         <is>
           <t>Item</t>
         </is>
       </c>
-      <c r="B4" s="12" t="inlineStr">
+      <c r="B4" s="13" t="inlineStr">
         <is>
           <t>Details</t>
         </is>
       </c>
     </row>
     <row r="5" ht="15" customHeight="1">
-      <c r="A5" s="13" t="inlineStr">
+      <c r="A5" s="14" t="inlineStr">
         <is>
           <t>Test Case ID</t>
         </is>
       </c>
-      <c r="B5" s="14" t="inlineStr">
+      <c r="B5" s="15" t="inlineStr">
         <is>
           <t>TC-013</t>
         </is>
       </c>
     </row>
     <row r="6" ht="15" customHeight="1">
-      <c r="A6" s="13" t="inlineStr">
+      <c r="A6" s="14" t="inlineStr">
         <is>
           <t>Test Scenario</t>
         </is>
       </c>
-      <c r="B6" s="14" t="inlineStr">
+      <c r="B6" s="15" t="inlineStr">
         <is>
           <t>Check an organiser sees only the events they organise</t>
         </is>
       </c>
     </row>
     <row r="7" ht="28" customHeight="1">
-      <c r="A7" s="13" t="inlineStr">
+      <c r="A7" s="14" t="inlineStr">
         <is>
           <t>Pre-conditions</t>
         </is>
       </c>
-      <c r="B7" s="14" t="inlineStr">
+      <c r="B7" s="15" t="inlineStr">
         <is>
           <t>App running (frontend http://localhost:3000, backend on shared Supabase DB). Page freshly loaded (seed event data). Account active and not locked.</t>
         </is>
       </c>
     </row>
     <row r="8" ht="28" customHeight="1">
-      <c r="A8" s="13" t="inlineStr">
+      <c r="A8" s="14" t="inlineStr">
         <is>
           <t>Test Steps</t>
         </is>
       </c>
-      <c r="B8" s="14" t="inlineStr">
+      <c r="B8" s="15" t="inlineStr">
         <is>
           <t>1. Log in as the organiser
 2. On My events, read the list of event requests</t>
@@ -1077,67 +1077,67 @@
       </c>
     </row>
     <row r="9" ht="15" customHeight="1">
-      <c r="A9" s="13" t="inlineStr">
+      <c r="A9" s="14" t="inlineStr">
         <is>
           <t>Test Data</t>
         </is>
       </c>
-      <c r="B9" s="14" t="inlineStr">
+      <c r="B9" s="15" t="inlineStr">
         <is>
           <t>Email=maya.rahman@connectsphere.edu; Password=&lt;team password&gt;</t>
         </is>
       </c>
     </row>
     <row r="10" ht="42" customHeight="1">
-      <c r="A10" s="13" t="inlineStr">
+      <c r="A10" s="14" t="inlineStr">
         <is>
           <t>Expected Result</t>
         </is>
       </c>
-      <c r="B10" s="14" t="inlineStr">
+      <c r="B10" s="15" t="inlineStr">
         <is>
           <t>Only Maya's events are listed: Alumni Homecoming Dinner, Design Week Keynote, Postgrad Mixer. Other organisers' events (e.g. Research Symposium - Day 1, Startup Pitch Night, Open House 2026) are not shown</t>
         </is>
       </c>
     </row>
     <row r="11" ht="15" customHeight="1">
-      <c r="A11" s="13" t="inlineStr">
+      <c r="A11" s="14" t="inlineStr">
         <is>
           <t>Created By</t>
         </is>
       </c>
-      <c r="B11" s="14" t="inlineStr">
+      <c r="B11" s="15" t="inlineStr">
         <is>
           <t>Zhenhan</t>
         </is>
       </c>
     </row>
     <row r="12" ht="15" customHeight="1">
-      <c r="A12" s="13" t="inlineStr">
+      <c r="A12" s="14" t="inlineStr">
         <is>
           <t>Date of Creation</t>
         </is>
       </c>
-      <c r="B12" s="14" t="inlineStr">
+      <c r="B12" s="15" t="inlineStr">
         <is>
           <t>06/10/2026</t>
         </is>
       </c>
     </row>
     <row r="13" ht="15" customHeight="1">
-      <c r="A13" s="15" t="inlineStr">
+      <c r="A13" s="16" t="inlineStr">
         <is>
           <t>Item</t>
         </is>
       </c>
-      <c r="B13" s="15" t="inlineStr">
+      <c r="B13" s="16" t="inlineStr">
         <is>
           <t>Details</t>
         </is>
       </c>
     </row>
     <row r="14" ht="28" customHeight="1">
-      <c r="A14" s="16" t="inlineStr">
+      <c r="A14" s="7" t="inlineStr">
         <is>
           <t>Actual Result</t>
         </is>
@@ -1149,7 +1149,7 @@
       </c>
     </row>
     <row r="15" ht="15" customHeight="1">
-      <c r="A15" s="16" t="inlineStr">
+      <c r="A15" s="7" t="inlineStr">
         <is>
           <t>Pass/Fail/Not Executed/Blocked</t>
         </is>
@@ -1161,7 +1161,7 @@
       </c>
     </row>
     <row r="16" ht="15" customHeight="1">
-      <c r="A16" s="16" t="inlineStr">
+      <c r="A16" s="7" t="inlineStr">
         <is>
           <t>Remarks</t>
         </is>
@@ -1173,7 +1173,7 @@
       </c>
     </row>
     <row r="17" ht="15" customHeight="1">
-      <c r="A17" s="16" t="inlineStr">
+      <c r="A17" s="7" t="inlineStr">
         <is>
           <t>Executed By</t>
         </is>
@@ -1185,7 +1185,7 @@
       </c>
     </row>
     <row r="18" ht="15" customHeight="1">
-      <c r="A18" s="16" t="inlineStr">
+      <c r="A18" s="7" t="inlineStr">
         <is>
           <t>Date of Execution</t>
         </is>
@@ -1197,60 +1197,60 @@
       </c>
     </row>
     <row r="21" ht="15" customHeight="1">
-      <c r="A21" s="12" t="inlineStr">
+      <c r="A21" s="13" t="inlineStr">
         <is>
           <t>Item</t>
         </is>
       </c>
-      <c r="B21" s="12" t="inlineStr">
+      <c r="B21" s="13" t="inlineStr">
         <is>
           <t>Details</t>
         </is>
       </c>
     </row>
     <row r="22" ht="15" customHeight="1">
-      <c r="A22" s="13" t="inlineStr">
+      <c r="A22" s="14" t="inlineStr">
         <is>
           <t>Test Case ID</t>
         </is>
       </c>
-      <c r="B22" s="14" t="inlineStr">
+      <c r="B22" s="15" t="inlineStr">
         <is>
           <t>TC-014</t>
         </is>
       </c>
     </row>
     <row r="23" ht="15" customHeight="1">
-      <c r="A23" s="13" t="inlineStr">
+      <c r="A23" s="14" t="inlineStr">
         <is>
           <t>Test Scenario</t>
         </is>
       </c>
-      <c r="B23" s="14" t="inlineStr">
-        <is>
-          <t>Check an attendee sees only published events open for registration</t>
+      <c r="B23" s="15" t="inlineStr">
+        <is>
+          <t>Check an attendee sees only confirmed events open for registration</t>
         </is>
       </c>
     </row>
     <row r="24" ht="28" customHeight="1">
-      <c r="A24" s="13" t="inlineStr">
+      <c r="A24" s="14" t="inlineStr">
         <is>
           <t>Pre-conditions</t>
         </is>
       </c>
-      <c r="B24" s="14" t="inlineStr">
+      <c r="B24" s="15" t="inlineStr">
         <is>
           <t>App running (frontend http://localhost:3000, backend on shared Supabase DB). Page freshly loaded (seed event data). Account active and not locked.</t>
         </is>
       </c>
     </row>
     <row r="25" ht="28" customHeight="1">
-      <c r="A25" s="13" t="inlineStr">
+      <c r="A25" s="14" t="inlineStr">
         <is>
           <t>Test Steps</t>
         </is>
       </c>
-      <c r="B25" s="14" t="inlineStr">
+      <c r="B25" s="15" t="inlineStr">
         <is>
           <t>1. Log in as the attendee
 2. On Browse events, read the list of events</t>
@@ -1258,103 +1258,103 @@
       </c>
     </row>
     <row r="26" ht="15" customHeight="1">
-      <c r="A26" s="13" t="inlineStr">
+      <c r="A26" s="14" t="inlineStr">
         <is>
           <t>Test Data</t>
         </is>
       </c>
-      <c r="B26" s="14" t="inlineStr">
+      <c r="B26" s="15" t="inlineStr">
         <is>
           <t>Email=sam.adeyemi@student.connectsphere.edu; Password=&lt;team password&gt;</t>
         </is>
       </c>
     </row>
     <row r="27" ht="42" customHeight="1">
-      <c r="A27" s="13" t="inlineStr">
+      <c r="A27" s="14" t="inlineStr">
         <is>
           <t>Expected Result</t>
         </is>
       </c>
-      <c r="B27" s="14" t="inlineStr">
-        <is>
-          <t>Only events in Planning/Confirmed with registration open are listed (Design Week Keynote, Industry Career Fair, Sustainability Forum, Open House 2026). Drafts and requests under review (e.g. Postgrad Mixer, Alumni Homecoming Dinner) are not shown</t>
+      <c r="B27" s="15" t="inlineStr">
+        <is>
+          <t>Only Confirmed events with registration open are listed (Open House 2026). Approved events still being arranged (e.g. Design Week Keynote, Industry Career Fair), drafts and requests under review (e.g. Postgrad Mixer, Alumni Homecoming Dinner) are not shown</t>
         </is>
       </c>
     </row>
     <row r="28" ht="15" customHeight="1">
-      <c r="A28" s="13" t="inlineStr">
+      <c r="A28" s="14" t="inlineStr">
         <is>
           <t>Created By</t>
         </is>
       </c>
-      <c r="B28" s="14" t="inlineStr">
+      <c r="B28" s="15" t="inlineStr">
         <is>
           <t>Zhenhan</t>
         </is>
       </c>
     </row>
     <row r="29" ht="15" customHeight="1">
-      <c r="A29" s="13" t="inlineStr">
+      <c r="A29" s="14" t="inlineStr">
         <is>
           <t>Date of Creation</t>
         </is>
       </c>
-      <c r="B29" s="14" t="inlineStr">
+      <c r="B29" s="15" t="inlineStr">
         <is>
           <t>06/10/2026</t>
         </is>
       </c>
     </row>
     <row r="30" ht="15" customHeight="1">
-      <c r="A30" s="15" t="inlineStr">
+      <c r="A30" s="16" t="inlineStr">
         <is>
           <t>Item</t>
         </is>
       </c>
-      <c r="B30" s="15" t="inlineStr">
+      <c r="B30" s="16" t="inlineStr">
         <is>
           <t>Details</t>
         </is>
       </c>
     </row>
-    <row r="31" ht="42" customHeight="1">
-      <c r="A31" s="16" t="inlineStr">
+    <row r="31" ht="28" customHeight="1">
+      <c r="A31" s="7" t="inlineStr">
         <is>
           <t>Actual Result</t>
         </is>
       </c>
       <c r="B31" s="17" t="inlineStr">
         <is>
-          <t>Browse events lists: Design Week Keynote, Industry Career Fair, Sustainability Forum, Open House 2026. Drafts / requests under review (Postgrad Mixer, Alumni Homecoming Dinner, Startup Pitch Night) hidden = True</t>
+          <t>Re-run needed. Previous run (06/10/2026) passed under the earlier rule, where Approved/Planning events were also published to attendees.</t>
         </is>
       </c>
     </row>
     <row r="32" ht="15" customHeight="1">
-      <c r="A32" s="16" t="inlineStr">
+      <c r="A32" s="7" t="inlineStr">
         <is>
           <t>Pass/Fail/Not Executed/Blocked</t>
         </is>
       </c>
-      <c r="B32" s="5" t="inlineStr">
-        <is>
-          <t>Pass</t>
-        </is>
-      </c>
-    </row>
-    <row r="33" ht="15" customHeight="1">
-      <c r="A33" s="16" t="inlineStr">
+      <c r="B32" s="7" t="inlineStr">
+        <is>
+          <t>Not Executed</t>
+        </is>
+      </c>
+    </row>
+    <row r="33" ht="42" customHeight="1">
+      <c r="A33" s="7" t="inlineStr">
         <is>
           <t>Remarks</t>
         </is>
       </c>
       <c r="B33" s="17" t="inlineStr">
         <is>
-          <t>NA</t>
+          <t>Rule changed 08/10/2026: attendees see only Confirmed events (an approved event's venue/date may still change). Covered by automated tests: tests/us02_rbac/event-visibility.unit.test.ts, tests/us03_us04_event_request/test_list_events.py.</t>
         </is>
       </c>
     </row>
     <row r="34" ht="15" customHeight="1">
-      <c r="A34" s="16" t="inlineStr">
+      <c r="A34" s="7" t="inlineStr">
         <is>
           <t>Executed By</t>
         </is>
@@ -1366,7 +1366,7 @@
       </c>
     </row>
     <row r="35" ht="15" customHeight="1">
-      <c r="A35" s="16" t="inlineStr">
+      <c r="A35" s="7" t="inlineStr">
         <is>
           <t>Date of Execution</t>
         </is>
@@ -1378,60 +1378,60 @@
       </c>
     </row>
     <row r="38" ht="15" customHeight="1">
-      <c r="A38" s="12" t="inlineStr">
+      <c r="A38" s="13" t="inlineStr">
         <is>
           <t>Item</t>
         </is>
       </c>
-      <c r="B38" s="12" t="inlineStr">
+      <c r="B38" s="13" t="inlineStr">
         <is>
           <t>Details</t>
         </is>
       </c>
     </row>
     <row r="39" ht="15" customHeight="1">
-      <c r="A39" s="13" t="inlineStr">
+      <c r="A39" s="14" t="inlineStr">
         <is>
           <t>Test Case ID</t>
         </is>
       </c>
-      <c r="B39" s="14" t="inlineStr">
+      <c r="B39" s="15" t="inlineStr">
         <is>
           <t>TC-015</t>
         </is>
       </c>
     </row>
     <row r="40" ht="15" customHeight="1">
-      <c r="A40" s="13" t="inlineStr">
+      <c r="A40" s="14" t="inlineStr">
         <is>
           <t>Test Scenario</t>
         </is>
       </c>
-      <c r="B40" s="14" t="inlineStr">
+      <c r="B40" s="15" t="inlineStr">
         <is>
           <t>Check a coordinator cannot see organisers' unsubmitted drafts</t>
         </is>
       </c>
     </row>
     <row r="41" ht="28" customHeight="1">
-      <c r="A41" s="13" t="inlineStr">
+      <c r="A41" s="14" t="inlineStr">
         <is>
           <t>Pre-conditions</t>
         </is>
       </c>
-      <c r="B41" s="14" t="inlineStr">
+      <c r="B41" s="15" t="inlineStr">
         <is>
           <t>App running (frontend http://localhost:3000, backend on shared Supabase DB). Page freshly loaded (seed event data). Account active and not locked.</t>
         </is>
       </c>
     </row>
     <row r="42" ht="42" customHeight="1">
-      <c r="A42" s="13" t="inlineStr">
+      <c r="A42" s="14" t="inlineStr">
         <is>
           <t>Test Steps</t>
         </is>
       </c>
-      <c r="B42" s="14" t="inlineStr">
+      <c r="B42" s="15" t="inlineStr">
         <is>
           <t>1. Log in as the coordinator
 2. On Review queue, select the 'All' filter
@@ -1440,67 +1440,67 @@
       </c>
     </row>
     <row r="43" ht="15" customHeight="1">
-      <c r="A43" s="13" t="inlineStr">
+      <c r="A43" s="14" t="inlineStr">
         <is>
           <t>Test Data</t>
         </is>
       </c>
-      <c r="B43" s="14" t="inlineStr">
+      <c r="B43" s="15" t="inlineStr">
         <is>
           <t>Email=priya.tan@connectsphere.edu; Password=&lt;team password&gt;</t>
         </is>
       </c>
     </row>
     <row r="44" ht="15" customHeight="1">
-      <c r="A44" s="13" t="inlineStr">
+      <c r="A44" s="14" t="inlineStr">
         <is>
           <t>Expected Result</t>
         </is>
       </c>
-      <c r="B44" s="14" t="inlineStr">
+      <c r="B44" s="15" t="inlineStr">
         <is>
           <t>Submitted / in-progress requests are listed; the draft 'Postgrad Mixer' is not shown</t>
         </is>
       </c>
     </row>
     <row r="45" ht="15" customHeight="1">
-      <c r="A45" s="13" t="inlineStr">
+      <c r="A45" s="14" t="inlineStr">
         <is>
           <t>Created By</t>
         </is>
       </c>
-      <c r="B45" s="14" t="inlineStr">
+      <c r="B45" s="15" t="inlineStr">
         <is>
           <t>Zhenhan</t>
         </is>
       </c>
     </row>
     <row r="46" ht="15" customHeight="1">
-      <c r="A46" s="13" t="inlineStr">
+      <c r="A46" s="14" t="inlineStr">
         <is>
           <t>Date of Creation</t>
         </is>
       </c>
-      <c r="B46" s="14" t="inlineStr">
+      <c r="B46" s="15" t="inlineStr">
         <is>
           <t>06/10/2026</t>
         </is>
       </c>
     </row>
     <row r="47" ht="15" customHeight="1">
-      <c r="A47" s="15" t="inlineStr">
+      <c r="A47" s="16" t="inlineStr">
         <is>
           <t>Item</t>
         </is>
       </c>
-      <c r="B47" s="15" t="inlineStr">
+      <c r="B47" s="16" t="inlineStr">
         <is>
           <t>Details</t>
         </is>
       </c>
     </row>
     <row r="48" ht="28" customHeight="1">
-      <c r="A48" s="16" t="inlineStr">
+      <c r="A48" s="7" t="inlineStr">
         <is>
           <t>Actual Result</t>
         </is>
@@ -1512,7 +1512,7 @@
       </c>
     </row>
     <row r="49" ht="15" customHeight="1">
-      <c r="A49" s="16" t="inlineStr">
+      <c r="A49" s="7" t="inlineStr">
         <is>
           <t>Pass/Fail/Not Executed/Blocked</t>
         </is>
@@ -1524,7 +1524,7 @@
       </c>
     </row>
     <row r="50" ht="15" customHeight="1">
-      <c r="A50" s="16" t="inlineStr">
+      <c r="A50" s="7" t="inlineStr">
         <is>
           <t>Remarks</t>
         </is>
@@ -1536,7 +1536,7 @@
       </c>
     </row>
     <row r="51" ht="15" customHeight="1">
-      <c r="A51" s="16" t="inlineStr">
+      <c r="A51" s="7" t="inlineStr">
         <is>
           <t>Executed By</t>
         </is>
@@ -1548,7 +1548,7 @@
       </c>
     </row>
     <row r="52" ht="15" customHeight="1">
-      <c r="A52" s="16" t="inlineStr">
+      <c r="A52" s="7" t="inlineStr">
         <is>
           <t>Date of Execution</t>
         </is>
@@ -1560,60 +1560,60 @@
       </c>
     </row>
     <row r="55" ht="15" customHeight="1">
-      <c r="A55" s="12" t="inlineStr">
+      <c r="A55" s="13" t="inlineStr">
         <is>
           <t>Item</t>
         </is>
       </c>
-      <c r="B55" s="12" t="inlineStr">
+      <c r="B55" s="13" t="inlineStr">
         <is>
           <t>Details</t>
         </is>
       </c>
     </row>
     <row r="56" ht="15" customHeight="1">
-      <c r="A56" s="13" t="inlineStr">
+      <c r="A56" s="14" t="inlineStr">
         <is>
           <t>Test Case ID</t>
         </is>
       </c>
-      <c r="B56" s="14" t="inlineStr">
+      <c r="B56" s="15" t="inlineStr">
         <is>
           <t>TC-016</t>
         </is>
       </c>
     </row>
     <row r="57" ht="15" customHeight="1">
-      <c r="A57" s="13" t="inlineStr">
+      <c r="A57" s="14" t="inlineStr">
         <is>
           <t>Test Scenario</t>
         </is>
       </c>
-      <c r="B57" s="14" t="inlineStr">
+      <c r="B57" s="15" t="inlineStr">
         <is>
           <t>Check each role's navigation shows only the pages for that role</t>
         </is>
       </c>
     </row>
     <row r="58" ht="28" customHeight="1">
-      <c r="A58" s="13" t="inlineStr">
+      <c r="A58" s="14" t="inlineStr">
         <is>
           <t>Pre-conditions</t>
         </is>
       </c>
-      <c r="B58" s="14" t="inlineStr">
+      <c r="B58" s="15" t="inlineStr">
         <is>
           <t>App running (frontend http://localhost:3000, backend on shared Supabase DB). Page freshly loaded (seed event data). Account active and not locked.</t>
         </is>
       </c>
     </row>
     <row r="59" ht="56" customHeight="1">
-      <c r="A59" s="13" t="inlineStr">
+      <c r="A59" s="14" t="inlineStr">
         <is>
           <t>Test Steps</t>
         </is>
       </c>
-      <c r="B59" s="14" t="inlineStr">
+      <c r="B59" s="15" t="inlineStr">
         <is>
           <t>1. Log in with the first account in Test Data
 2. Note the items in the sidebar
@@ -1623,67 +1623,67 @@
       </c>
     </row>
     <row r="60" ht="28" customHeight="1">
-      <c r="A60" s="13" t="inlineStr">
+      <c r="A60" s="14" t="inlineStr">
         <is>
           <t>Test Data</t>
         </is>
       </c>
-      <c r="B60" s="14" t="inlineStr">
+      <c r="B60" s="15" t="inlineStr">
         <is>
           <t>maya.rahman@connectsphere.edu; priya.tan@connectsphere.edu; daniel.ortiz@connectsphere.edu; wei.lim@connectsphere.edu; sam.adeyemi@student.connectsphere.edu; Password=&lt;team password&gt;</t>
         </is>
       </c>
     </row>
     <row r="61" ht="42" customHeight="1">
-      <c r="A61" s="13" t="inlineStr">
+      <c r="A61" s="14" t="inlineStr">
         <is>
           <t>Expected Result</t>
         </is>
       </c>
-      <c r="B61" s="14" t="inlineStr">
+      <c r="B61" s="15" t="inlineStr">
         <is>
           <t>Organiser: My events, New request. Coordinator: Review queue, Pipeline. Venue Staff: Booking requests, Venue catalogue. Technical Support: Equipment. Attendee: Browse events. No other pages listed</t>
         </is>
       </c>
     </row>
     <row r="62" ht="15" customHeight="1">
-      <c r="A62" s="13" t="inlineStr">
+      <c r="A62" s="14" t="inlineStr">
         <is>
           <t>Created By</t>
         </is>
       </c>
-      <c r="B62" s="14" t="inlineStr">
+      <c r="B62" s="15" t="inlineStr">
         <is>
           <t>Zhenhan</t>
         </is>
       </c>
     </row>
     <row r="63" ht="15" customHeight="1">
-      <c r="A63" s="13" t="inlineStr">
+      <c r="A63" s="14" t="inlineStr">
         <is>
           <t>Date of Creation</t>
         </is>
       </c>
-      <c r="B63" s="14" t="inlineStr">
+      <c r="B63" s="15" t="inlineStr">
         <is>
           <t>06/10/2026</t>
         </is>
       </c>
     </row>
     <row r="64" ht="15" customHeight="1">
-      <c r="A64" s="15" t="inlineStr">
+      <c r="A64" s="16" t="inlineStr">
         <is>
           <t>Item</t>
         </is>
       </c>
-      <c r="B64" s="15" t="inlineStr">
+      <c r="B64" s="16" t="inlineStr">
         <is>
           <t>Details</t>
         </is>
       </c>
     </row>
     <row r="65" ht="28" customHeight="1">
-      <c r="A65" s="16" t="inlineStr">
+      <c r="A65" s="7" t="inlineStr">
         <is>
           <t>Actual Result</t>
         </is>
@@ -1695,7 +1695,7 @@
       </c>
     </row>
     <row r="66" ht="15" customHeight="1">
-      <c r="A66" s="16" t="inlineStr">
+      <c r="A66" s="7" t="inlineStr">
         <is>
           <t>Pass/Fail/Not Executed/Blocked</t>
         </is>
@@ -1707,7 +1707,7 @@
       </c>
     </row>
     <row r="67" ht="15" customHeight="1">
-      <c r="A67" s="16" t="inlineStr">
+      <c r="A67" s="7" t="inlineStr">
         <is>
           <t>Remarks</t>
         </is>
@@ -1719,7 +1719,7 @@
       </c>
     </row>
     <row r="68" ht="15" customHeight="1">
-      <c r="A68" s="16" t="inlineStr">
+      <c r="A68" s="7" t="inlineStr">
         <is>
           <t>Executed By</t>
         </is>
@@ -1731,7 +1731,7 @@
       </c>
     </row>
     <row r="69" ht="15" customHeight="1">
-      <c r="A69" s="16" t="inlineStr">
+      <c r="A69" s="7" t="inlineStr">
         <is>
           <t>Date of Execution</t>
         </is>
@@ -1743,60 +1743,60 @@
       </c>
     </row>
     <row r="72" ht="15" customHeight="1">
-      <c r="A72" s="12" t="inlineStr">
+      <c r="A72" s="13" t="inlineStr">
         <is>
           <t>Item</t>
         </is>
       </c>
-      <c r="B72" s="12" t="inlineStr">
+      <c r="B72" s="13" t="inlineStr">
         <is>
           <t>Details</t>
         </is>
       </c>
     </row>
     <row r="73" ht="15" customHeight="1">
-      <c r="A73" s="13" t="inlineStr">
+      <c r="A73" s="14" t="inlineStr">
         <is>
           <t>Test Case ID</t>
         </is>
       </c>
-      <c r="B73" s="14" t="inlineStr">
+      <c r="B73" s="15" t="inlineStr">
         <is>
           <t>TC-017</t>
         </is>
       </c>
     </row>
     <row r="74" ht="15" customHeight="1">
-      <c r="A74" s="13" t="inlineStr">
+      <c r="A74" s="14" t="inlineStr">
         <is>
           <t>Test Scenario</t>
         </is>
       </c>
-      <c r="B74" s="14" t="inlineStr">
+      <c r="B74" s="15" t="inlineStr">
         <is>
           <t>Check a user cannot open another role's page by typing its URL</t>
         </is>
       </c>
     </row>
     <row r="75" ht="28" customHeight="1">
-      <c r="A75" s="13" t="inlineStr">
+      <c r="A75" s="14" t="inlineStr">
         <is>
           <t>Pre-conditions</t>
         </is>
       </c>
-      <c r="B75" s="14" t="inlineStr">
+      <c r="B75" s="15" t="inlineStr">
         <is>
           <t>App running (frontend http://localhost:3000, backend on shared Supabase DB). Page freshly loaded (seed event data). Account active and not locked.</t>
         </is>
       </c>
     </row>
     <row r="76" ht="42" customHeight="1">
-      <c r="A76" s="13" t="inlineStr">
+      <c r="A76" s="14" t="inlineStr">
         <is>
           <t>Test Steps</t>
         </is>
       </c>
-      <c r="B76" s="14" t="inlineStr">
+      <c r="B76" s="15" t="inlineStr">
         <is>
           <t>1. Log in as the organiser
 2. Type http://localhost:3000/queue in the address bar and press Enter
@@ -1805,67 +1805,67 @@
       </c>
     </row>
     <row r="77" ht="28" customHeight="1">
-      <c r="A77" s="13" t="inlineStr">
+      <c r="A77" s="14" t="inlineStr">
         <is>
           <t>Test Data</t>
         </is>
       </c>
-      <c r="B77" s="14" t="inlineStr">
+      <c r="B77" s="15" t="inlineStr">
         <is>
           <t>Email=maya.rahman@connectsphere.edu; Password=&lt;team password&gt;; URLs=/queue, /catalogue, /equipment</t>
         </is>
       </c>
     </row>
     <row r="78" ht="28" customHeight="1">
-      <c r="A78" s="13" t="inlineStr">
+      <c r="A78" s="14" t="inlineStr">
         <is>
           <t>Expected Result</t>
         </is>
       </c>
-      <c r="B78" s="14" t="inlineStr">
+      <c r="B78" s="15" t="inlineStr">
         <is>
           <t>The other role's page is never displayed; user is returned to My events and shown an authorisation message (e.g. 'You don't have permission to view that page')</t>
         </is>
       </c>
     </row>
     <row r="79" ht="15" customHeight="1">
-      <c r="A79" s="13" t="inlineStr">
+      <c r="A79" s="14" t="inlineStr">
         <is>
           <t>Created By</t>
         </is>
       </c>
-      <c r="B79" s="14" t="inlineStr">
+      <c r="B79" s="15" t="inlineStr">
         <is>
           <t>Zhenhan</t>
         </is>
       </c>
     </row>
     <row r="80" ht="15" customHeight="1">
-      <c r="A80" s="13" t="inlineStr">
+      <c r="A80" s="14" t="inlineStr">
         <is>
           <t>Date of Creation</t>
         </is>
       </c>
-      <c r="B80" s="14" t="inlineStr">
+      <c r="B80" s="15" t="inlineStr">
         <is>
           <t>06/10/2026</t>
         </is>
       </c>
     </row>
     <row r="81" ht="15" customHeight="1">
-      <c r="A81" s="15" t="inlineStr">
+      <c r="A81" s="16" t="inlineStr">
         <is>
           <t>Item</t>
         </is>
       </c>
-      <c r="B81" s="15" t="inlineStr">
+      <c r="B81" s="16" t="inlineStr">
         <is>
           <t>Details</t>
         </is>
       </c>
     </row>
     <row r="82" ht="56" customHeight="1">
-      <c r="A82" s="16" t="inlineStr">
+      <c r="A82" s="7" t="inlineStr">
         <is>
           <t>Actual Result</t>
         </is>
@@ -1877,7 +1877,7 @@
       </c>
     </row>
     <row r="83" ht="15" customHeight="1">
-      <c r="A83" s="16" t="inlineStr">
+      <c r="A83" s="7" t="inlineStr">
         <is>
           <t>Pass/Fail/Not Executed/Blocked</t>
         </is>
@@ -1889,7 +1889,7 @@
       </c>
     </row>
     <row r="84" ht="15" customHeight="1">
-      <c r="A84" s="16" t="inlineStr">
+      <c r="A84" s="7" t="inlineStr">
         <is>
           <t>Remarks</t>
         </is>
@@ -1901,7 +1901,7 @@
       </c>
     </row>
     <row r="85" ht="15" customHeight="1">
-      <c r="A85" s="16" t="inlineStr">
+      <c r="A85" s="7" t="inlineStr">
         <is>
           <t>Executed By</t>
         </is>
@@ -1913,7 +1913,7 @@
       </c>
     </row>
     <row r="86" ht="15" customHeight="1">
-      <c r="A86" s="16" t="inlineStr">
+      <c r="A86" s="7" t="inlineStr">
         <is>
           <t>Date of Execution</t>
         </is>
@@ -1925,60 +1925,60 @@
       </c>
     </row>
     <row r="89" ht="15" customHeight="1">
-      <c r="A89" s="12" t="inlineStr">
+      <c r="A89" s="13" t="inlineStr">
         <is>
           <t>Item</t>
         </is>
       </c>
-      <c r="B89" s="12" t="inlineStr">
+      <c r="B89" s="13" t="inlineStr">
         <is>
           <t>Details</t>
         </is>
       </c>
     </row>
     <row r="90" ht="15" customHeight="1">
-      <c r="A90" s="13" t="inlineStr">
+      <c r="A90" s="14" t="inlineStr">
         <is>
           <t>Test Case ID</t>
         </is>
       </c>
-      <c r="B90" s="14" t="inlineStr">
+      <c r="B90" s="15" t="inlineStr">
         <is>
           <t>TC-018</t>
         </is>
       </c>
     </row>
     <row r="91" ht="15" customHeight="1">
-      <c r="A91" s="13" t="inlineStr">
+      <c r="A91" s="14" t="inlineStr">
         <is>
           <t>Test Scenario</t>
         </is>
       </c>
-      <c r="B91" s="14" t="inlineStr">
+      <c r="B91" s="15" t="inlineStr">
         <is>
           <t>Check a signed-out user cannot open any protected page</t>
         </is>
       </c>
     </row>
     <row r="92" ht="15" customHeight="1">
-      <c r="A92" s="13" t="inlineStr">
+      <c r="A92" s="14" t="inlineStr">
         <is>
           <t>Pre-conditions</t>
         </is>
       </c>
-      <c r="B92" s="14" t="inlineStr">
+      <c r="B92" s="15" t="inlineStr">
         <is>
           <t>App running. User is signed out.</t>
         </is>
       </c>
     </row>
     <row r="93" ht="28" customHeight="1">
-      <c r="A93" s="13" t="inlineStr">
+      <c r="A93" s="14" t="inlineStr">
         <is>
           <t>Test Steps</t>
         </is>
       </c>
-      <c r="B93" s="14" t="inlineStr">
+      <c r="B93" s="15" t="inlineStr">
         <is>
           <t>1. Type http://localhost:3000/my-events in the address bar and press Enter
 2. Repeat with /queue and /catalogue</t>
@@ -1986,67 +1986,67 @@
       </c>
     </row>
     <row r="94" ht="15" customHeight="1">
-      <c r="A94" s="13" t="inlineStr">
+      <c r="A94" s="14" t="inlineStr">
         <is>
           <t>Test Data</t>
         </is>
       </c>
-      <c r="B94" s="14" t="inlineStr">
+      <c r="B94" s="15" t="inlineStr">
         <is>
           <t>URLs=/my-events, /queue, /catalogue</t>
         </is>
       </c>
     </row>
     <row r="95" ht="15" customHeight="1">
-      <c r="A95" s="13" t="inlineStr">
+      <c r="A95" s="14" t="inlineStr">
         <is>
           <t>Expected Result</t>
         </is>
       </c>
-      <c r="B95" s="14" t="inlineStr">
+      <c r="B95" s="15" t="inlineStr">
         <is>
           <t>Each time the user is sent to the login page; no event or venue data is displayed</t>
         </is>
       </c>
     </row>
     <row r="96" ht="15" customHeight="1">
-      <c r="A96" s="13" t="inlineStr">
+      <c r="A96" s="14" t="inlineStr">
         <is>
           <t>Created By</t>
         </is>
       </c>
-      <c r="B96" s="14" t="inlineStr">
+      <c r="B96" s="15" t="inlineStr">
         <is>
           <t>Zhenhan</t>
         </is>
       </c>
     </row>
     <row r="97" ht="15" customHeight="1">
-      <c r="A97" s="13" t="inlineStr">
+      <c r="A97" s="14" t="inlineStr">
         <is>
           <t>Date of Creation</t>
         </is>
       </c>
-      <c r="B97" s="14" t="inlineStr">
+      <c r="B97" s="15" t="inlineStr">
         <is>
           <t>06/10/2026</t>
         </is>
       </c>
     </row>
     <row r="98" ht="15" customHeight="1">
-      <c r="A98" s="15" t="inlineStr">
+      <c r="A98" s="16" t="inlineStr">
         <is>
           <t>Item</t>
         </is>
       </c>
-      <c r="B98" s="15" t="inlineStr">
+      <c r="B98" s="16" t="inlineStr">
         <is>
           <t>Details</t>
         </is>
       </c>
     </row>
     <row r="99" ht="28" customHeight="1">
-      <c r="A99" s="16" t="inlineStr">
+      <c r="A99" s="7" t="inlineStr">
         <is>
           <t>Actual Result</t>
         </is>
@@ -2058,7 +2058,7 @@
       </c>
     </row>
     <row r="100" ht="15" customHeight="1">
-      <c r="A100" s="16" t="inlineStr">
+      <c r="A100" s="7" t="inlineStr">
         <is>
           <t>Pass/Fail/Not Executed/Blocked</t>
         </is>
@@ -2070,7 +2070,7 @@
       </c>
     </row>
     <row r="101" ht="15" customHeight="1">
-      <c r="A101" s="16" t="inlineStr">
+      <c r="A101" s="7" t="inlineStr">
         <is>
           <t>Remarks</t>
         </is>
@@ -2082,7 +2082,7 @@
       </c>
     </row>
     <row r="102" ht="15" customHeight="1">
-      <c r="A102" s="16" t="inlineStr">
+      <c r="A102" s="7" t="inlineStr">
         <is>
           <t>Executed By</t>
         </is>
@@ -2094,7 +2094,7 @@
       </c>
     </row>
     <row r="103" ht="15" customHeight="1">
-      <c r="A103" s="16" t="inlineStr">
+      <c r="A103" s="7" t="inlineStr">
         <is>
           <t>Date of Execution</t>
         </is>
@@ -2106,60 +2106,60 @@
       </c>
     </row>
     <row r="106" ht="15" customHeight="1">
-      <c r="A106" s="12" t="inlineStr">
+      <c r="A106" s="13" t="inlineStr">
         <is>
           <t>Item</t>
         </is>
       </c>
-      <c r="B106" s="12" t="inlineStr">
+      <c r="B106" s="13" t="inlineStr">
         <is>
           <t>Details</t>
         </is>
       </c>
     </row>
     <row r="107" ht="15" customHeight="1">
-      <c r="A107" s="13" t="inlineStr">
+      <c r="A107" s="14" t="inlineStr">
         <is>
           <t>Test Case ID</t>
         </is>
       </c>
-      <c r="B107" s="14" t="inlineStr">
+      <c r="B107" s="15" t="inlineStr">
         <is>
           <t>TC-019</t>
         </is>
       </c>
     </row>
     <row r="108" ht="15" customHeight="1">
-      <c r="A108" s="13" t="inlineStr">
+      <c r="A108" s="14" t="inlineStr">
         <is>
           <t>Test Scenario</t>
         </is>
       </c>
-      <c r="B108" s="14" t="inlineStr">
+      <c r="B108" s="15" t="inlineStr">
         <is>
           <t>Check venue staff can perform a permitted action (edit a venue)</t>
         </is>
       </c>
     </row>
     <row r="109" ht="28" customHeight="1">
-      <c r="A109" s="13" t="inlineStr">
+      <c r="A109" s="14" t="inlineStr">
         <is>
           <t>Pre-conditions</t>
         </is>
       </c>
-      <c r="B109" s="14" t="inlineStr">
+      <c r="B109" s="15" t="inlineStr">
         <is>
           <t>App running (frontend http://localhost:3000, backend on shared Supabase DB). Page freshly loaded (seed event data). Account active and not locked.</t>
         </is>
       </c>
     </row>
     <row r="110" ht="70" customHeight="1">
-      <c r="A110" s="13" t="inlineStr">
+      <c r="A110" s="14" t="inlineStr">
         <is>
           <t>Test Steps</t>
         </is>
       </c>
-      <c r="B110" s="14" t="inlineStr">
+      <c r="B110" s="15" t="inlineStr">
         <is>
           <t>1. Log in as venue staff
 2. Open Venue catalogue
@@ -2170,67 +2170,67 @@
       </c>
     </row>
     <row r="111" ht="28" customHeight="1">
-      <c r="A111" s="13" t="inlineStr">
+      <c r="A111" s="14" t="inlineStr">
         <is>
           <t>Test Data</t>
         </is>
       </c>
-      <c r="B111" s="14" t="inlineStr">
+      <c r="B111" s="15" t="inlineStr">
         <is>
           <t>Email=daniel.ortiz@connectsphere.edu; Password=&lt;team password&gt;; Venue=first venue in the catalogue; Capacity=original + 1 (then restore)</t>
         </is>
       </c>
     </row>
     <row r="112" ht="28" customHeight="1">
-      <c r="A112" s="13" t="inlineStr">
+      <c r="A112" s="14" t="inlineStr">
         <is>
           <t>Expected Result</t>
         </is>
       </c>
-      <c r="B112" s="14" t="inlineStr">
+      <c r="B112" s="15" t="inlineStr">
         <is>
           <t>Save succeeds; after reload the venue shows the new capacity. Original value restored in step 5</t>
         </is>
       </c>
     </row>
     <row r="113" ht="15" customHeight="1">
-      <c r="A113" s="13" t="inlineStr">
+      <c r="A113" s="14" t="inlineStr">
         <is>
           <t>Created By</t>
         </is>
       </c>
-      <c r="B113" s="14" t="inlineStr">
+      <c r="B113" s="15" t="inlineStr">
         <is>
           <t>Zhenhan</t>
         </is>
       </c>
     </row>
     <row r="114" ht="15" customHeight="1">
-      <c r="A114" s="13" t="inlineStr">
+      <c r="A114" s="14" t="inlineStr">
         <is>
           <t>Date of Creation</t>
         </is>
       </c>
-      <c r="B114" s="14" t="inlineStr">
+      <c r="B114" s="15" t="inlineStr">
         <is>
           <t>06/10/2026</t>
         </is>
       </c>
     </row>
     <row r="115" ht="15" customHeight="1">
-      <c r="A115" s="15" t="inlineStr">
+      <c r="A115" s="16" t="inlineStr">
         <is>
           <t>Item</t>
         </is>
       </c>
-      <c r="B115" s="15" t="inlineStr">
+      <c r="B115" s="16" t="inlineStr">
         <is>
           <t>Details</t>
         </is>
       </c>
     </row>
     <row r="116" ht="28" customHeight="1">
-      <c r="A116" s="16" t="inlineStr">
+      <c r="A116" s="7" t="inlineStr">
         <is>
           <t>Actual Result</t>
         </is>
@@ -2242,7 +2242,7 @@
       </c>
     </row>
     <row r="117" ht="15" customHeight="1">
-      <c r="A117" s="16" t="inlineStr">
+      <c r="A117" s="7" t="inlineStr">
         <is>
           <t>Pass/Fail/Not Executed/Blocked</t>
         </is>
@@ -2254,7 +2254,7 @@
       </c>
     </row>
     <row r="118" ht="28" customHeight="1">
-      <c r="A118" s="16" t="inlineStr">
+      <c r="A118" s="7" t="inlineStr">
         <is>
           <t>Remarks</t>
         </is>
@@ -2266,7 +2266,7 @@
       </c>
     </row>
     <row r="119" ht="15" customHeight="1">
-      <c r="A119" s="16" t="inlineStr">
+      <c r="A119" s="7" t="inlineStr">
         <is>
           <t>Executed By</t>
         </is>
@@ -2278,7 +2278,7 @@
       </c>
     </row>
     <row r="120" ht="15" customHeight="1">
-      <c r="A120" s="16" t="inlineStr">
+      <c r="A120" s="7" t="inlineStr">
         <is>
           <t>Date of Execution</t>
         </is>
@@ -2290,60 +2290,60 @@
       </c>
     </row>
     <row r="123" ht="15" customHeight="1">
-      <c r="A123" s="12" t="inlineStr">
+      <c r="A123" s="13" t="inlineStr">
         <is>
           <t>Item</t>
         </is>
       </c>
-      <c r="B123" s="12" t="inlineStr">
+      <c r="B123" s="13" t="inlineStr">
         <is>
           <t>Details</t>
         </is>
       </c>
     </row>
     <row r="124" ht="15" customHeight="1">
-      <c r="A124" s="13" t="inlineStr">
+      <c r="A124" s="14" t="inlineStr">
         <is>
           <t>Test Case ID</t>
         </is>
       </c>
-      <c r="B124" s="14" t="inlineStr">
+      <c r="B124" s="15" t="inlineStr">
         <is>
           <t>TC-020</t>
         </is>
       </c>
     </row>
     <row r="125" ht="15" customHeight="1">
-      <c r="A125" s="13" t="inlineStr">
+      <c r="A125" s="14" t="inlineStr">
         <is>
           <t>Test Scenario</t>
         </is>
       </c>
-      <c r="B125" s="14" t="inlineStr">
+      <c r="B125" s="15" t="inlineStr">
         <is>
           <t>Check the server rejects creating a venue by a role that is not venue staff</t>
         </is>
       </c>
     </row>
     <row r="126" ht="28" customHeight="1">
-      <c r="A126" s="13" t="inlineStr">
+      <c r="A126" s="14" t="inlineStr">
         <is>
           <t>Pre-conditions</t>
         </is>
       </c>
-      <c r="B126" s="14" t="inlineStr">
+      <c r="B126" s="15" t="inlineStr">
         <is>
           <t>App running (frontend http://localhost:3000, backend on shared Supabase DB). Page freshly loaded (seed event data). Account active and not locked.</t>
         </is>
       </c>
     </row>
     <row r="127" ht="70" customHeight="1">
-      <c r="A127" s="13" t="inlineStr">
+      <c r="A127" s="14" t="inlineStr">
         <is>
           <t>Test Steps</t>
         </is>
       </c>
-      <c r="B127" s="14" t="inlineStr">
+      <c r="B127" s="15" t="inlineStr">
         <is>
           <t>1. Log in as the organiser
 2. Open DevTools (F12) &gt; Console and run:
@@ -2353,67 +2353,67 @@
       </c>
     </row>
     <row r="128" ht="15" customHeight="1">
-      <c r="A128" s="13" t="inlineStr">
+      <c r="A128" s="14" t="inlineStr">
         <is>
           <t>Test Data</t>
         </is>
       </c>
-      <c r="B128" s="14" t="inlineStr">
+      <c r="B128" s="15" t="inlineStr">
         <is>
           <t>Email=maya.rahman@connectsphere.edu; Password=&lt;team password&gt;; Venue name=RBAC Test Room</t>
         </is>
       </c>
     </row>
     <row r="129" ht="28" customHeight="1">
-      <c r="A129" s="13" t="inlineStr">
+      <c r="A129" s="14" t="inlineStr">
         <is>
           <t>Expected Result</t>
         </is>
       </c>
-      <c r="B129" s="14" t="inlineStr">
+      <c r="B129" s="15" t="inlineStr">
         <is>
           <t>Step 2 returns 403 ('You don't have permission to do that'); step 3: no venue named 'RBAC Test Room' exists</t>
         </is>
       </c>
     </row>
     <row r="130" ht="15" customHeight="1">
-      <c r="A130" s="13" t="inlineStr">
+      <c r="A130" s="14" t="inlineStr">
         <is>
           <t>Created By</t>
         </is>
       </c>
-      <c r="B130" s="14" t="inlineStr">
+      <c r="B130" s="15" t="inlineStr">
         <is>
           <t>Zhenhan</t>
         </is>
       </c>
     </row>
     <row r="131" ht="15" customHeight="1">
-      <c r="A131" s="13" t="inlineStr">
+      <c r="A131" s="14" t="inlineStr">
         <is>
           <t>Date of Creation</t>
         </is>
       </c>
-      <c r="B131" s="14" t="inlineStr">
+      <c r="B131" s="15" t="inlineStr">
         <is>
           <t>06/10/2026</t>
         </is>
       </c>
     </row>
     <row r="132" ht="15" customHeight="1">
-      <c r="A132" s="15" t="inlineStr">
+      <c r="A132" s="16" t="inlineStr">
         <is>
           <t>Item</t>
         </is>
       </c>
-      <c r="B132" s="15" t="inlineStr">
+      <c r="B132" s="16" t="inlineStr">
         <is>
           <t>Details</t>
         </is>
       </c>
     </row>
     <row r="133" ht="28" customHeight="1">
-      <c r="A133" s="16" t="inlineStr">
+      <c r="A133" s="7" t="inlineStr">
         <is>
           <t>Actual Result</t>
         </is>
@@ -2425,7 +2425,7 @@
       </c>
     </row>
     <row r="134" ht="15" customHeight="1">
-      <c r="A134" s="16" t="inlineStr">
+      <c r="A134" s="7" t="inlineStr">
         <is>
           <t>Pass/Fail/Not Executed/Blocked</t>
         </is>
@@ -2437,7 +2437,7 @@
       </c>
     </row>
     <row r="135" ht="15" customHeight="1">
-      <c r="A135" s="16" t="inlineStr">
+      <c r="A135" s="7" t="inlineStr">
         <is>
           <t>Remarks</t>
         </is>
@@ -2449,7 +2449,7 @@
       </c>
     </row>
     <row r="136" ht="15" customHeight="1">
-      <c r="A136" s="16" t="inlineStr">
+      <c r="A136" s="7" t="inlineStr">
         <is>
           <t>Executed By</t>
         </is>
@@ -2461,7 +2461,7 @@
       </c>
     </row>
     <row r="137" ht="15" customHeight="1">
-      <c r="A137" s="16" t="inlineStr">
+      <c r="A137" s="7" t="inlineStr">
         <is>
           <t>Date of Execution</t>
         </is>
@@ -2473,60 +2473,60 @@
       </c>
     </row>
     <row r="140" ht="15" customHeight="1">
-      <c r="A140" s="12" t="inlineStr">
+      <c r="A140" s="13" t="inlineStr">
         <is>
           <t>Item</t>
         </is>
       </c>
-      <c r="B140" s="12" t="inlineStr">
+      <c r="B140" s="13" t="inlineStr">
         <is>
           <t>Details</t>
         </is>
       </c>
     </row>
     <row r="141" ht="15" customHeight="1">
-      <c r="A141" s="13" t="inlineStr">
+      <c r="A141" s="14" t="inlineStr">
         <is>
           <t>Test Case ID</t>
         </is>
       </c>
-      <c r="B141" s="14" t="inlineStr">
+      <c r="B141" s="15" t="inlineStr">
         <is>
           <t>TC-021</t>
         </is>
       </c>
     </row>
     <row r="142" ht="15" customHeight="1">
-      <c r="A142" s="13" t="inlineStr">
+      <c r="A142" s="14" t="inlineStr">
         <is>
           <t>Test Scenario</t>
         </is>
       </c>
-      <c r="B142" s="14" t="inlineStr">
+      <c r="B142" s="15" t="inlineStr">
         <is>
           <t>Check the server rejects deactivating a venue by a role that is not venue staff</t>
         </is>
       </c>
     </row>
     <row r="143" ht="28" customHeight="1">
-      <c r="A143" s="13" t="inlineStr">
+      <c r="A143" s="14" t="inlineStr">
         <is>
           <t>Pre-conditions</t>
         </is>
       </c>
-      <c r="B143" s="14" t="inlineStr">
+      <c r="B143" s="15" t="inlineStr">
         <is>
           <t>App running (frontend http://localhost:3000, backend on shared Supabase DB). Page freshly loaded (seed event data). Account active and not locked.</t>
         </is>
       </c>
     </row>
     <row r="144" ht="70" customHeight="1">
-      <c r="A144" s="13" t="inlineStr">
+      <c r="A144" s="14" t="inlineStr">
         <is>
           <t>Test Steps</t>
         </is>
       </c>
-      <c r="B144" s="14" t="inlineStr">
+      <c r="B144" s="15" t="inlineStr">
         <is>
           <t>1. Log in as technical support
 2. Open DevTools (F12) &gt; Console and run:
@@ -2536,67 +2536,67 @@
       </c>
     </row>
     <row r="145" ht="28" customHeight="1">
-      <c r="A145" s="13" t="inlineStr">
+      <c r="A145" s="14" t="inlineStr">
         <is>
           <t>Test Data</t>
         </is>
       </c>
-      <c r="B145" s="14" t="inlineStr">
+      <c r="B145" s="15" t="inlineStr">
         <is>
           <t>Email=wei.lim@connectsphere.edu; Password=&lt;team password&gt;; Venue id=1 (use the id of any active venue)</t>
         </is>
       </c>
     </row>
     <row r="146" ht="28" customHeight="1">
-      <c r="A146" s="13" t="inlineStr">
+      <c r="A146" s="14" t="inlineStr">
         <is>
           <t>Expected Result</t>
         </is>
       </c>
-      <c r="B146" s="14" t="inlineStr">
+      <c r="B146" s="15" t="inlineStr">
         <is>
           <t>Step 2 returns 403 ('You don't have permission to do that'); step 3: the venue is still listed as active</t>
         </is>
       </c>
     </row>
     <row r="147" ht="15" customHeight="1">
-      <c r="A147" s="13" t="inlineStr">
+      <c r="A147" s="14" t="inlineStr">
         <is>
           <t>Created By</t>
         </is>
       </c>
-      <c r="B147" s="14" t="inlineStr">
+      <c r="B147" s="15" t="inlineStr">
         <is>
           <t>Zhenhan</t>
         </is>
       </c>
     </row>
     <row r="148" ht="15" customHeight="1">
-      <c r="A148" s="13" t="inlineStr">
+      <c r="A148" s="14" t="inlineStr">
         <is>
           <t>Date of Creation</t>
         </is>
       </c>
-      <c r="B148" s="14" t="inlineStr">
+      <c r="B148" s="15" t="inlineStr">
         <is>
           <t>06/10/2026</t>
         </is>
       </c>
     </row>
     <row r="149" ht="15" customHeight="1">
-      <c r="A149" s="15" t="inlineStr">
+      <c r="A149" s="16" t="inlineStr">
         <is>
           <t>Item</t>
         </is>
       </c>
-      <c r="B149" s="15" t="inlineStr">
+      <c r="B149" s="16" t="inlineStr">
         <is>
           <t>Details</t>
         </is>
       </c>
     </row>
     <row r="150" ht="28" customHeight="1">
-      <c r="A150" s="16" t="inlineStr">
+      <c r="A150" s="7" t="inlineStr">
         <is>
           <t>Actual Result</t>
         </is>
@@ -2608,7 +2608,7 @@
       </c>
     </row>
     <row r="151" ht="15" customHeight="1">
-      <c r="A151" s="16" t="inlineStr">
+      <c r="A151" s="7" t="inlineStr">
         <is>
           <t>Pass/Fail/Not Executed/Blocked</t>
         </is>
@@ -2620,7 +2620,7 @@
       </c>
     </row>
     <row r="152" ht="15" customHeight="1">
-      <c r="A152" s="16" t="inlineStr">
+      <c r="A152" s="7" t="inlineStr">
         <is>
           <t>Remarks</t>
         </is>
@@ -2632,7 +2632,7 @@
       </c>
     </row>
     <row r="153" ht="15" customHeight="1">
-      <c r="A153" s="16" t="inlineStr">
+      <c r="A153" s="7" t="inlineStr">
         <is>
           <t>Executed By</t>
         </is>
@@ -2644,7 +2644,7 @@
       </c>
     </row>
     <row r="154" ht="15" customHeight="1">
-      <c r="A154" s="16" t="inlineStr">
+      <c r="A154" s="7" t="inlineStr">
         <is>
           <t>Date of Execution</t>
         </is>
@@ -2656,60 +2656,60 @@
       </c>
     </row>
     <row r="157" ht="15" customHeight="1">
-      <c r="A157" s="12" t="inlineStr">
+      <c r="A157" s="13" t="inlineStr">
         <is>
           <t>Item</t>
         </is>
       </c>
-      <c r="B157" s="12" t="inlineStr">
+      <c r="B157" s="13" t="inlineStr">
         <is>
           <t>Details</t>
         </is>
       </c>
     </row>
     <row r="158" ht="15" customHeight="1">
-      <c r="A158" s="13" t="inlineStr">
+      <c r="A158" s="14" t="inlineStr">
         <is>
           <t>Test Case ID</t>
         </is>
       </c>
-      <c r="B158" s="14" t="inlineStr">
+      <c r="B158" s="15" t="inlineStr">
         <is>
           <t>TC-022</t>
         </is>
       </c>
     </row>
     <row r="159" ht="15" customHeight="1">
-      <c r="A159" s="13" t="inlineStr">
+      <c r="A159" s="14" t="inlineStr">
         <is>
           <t>Test Scenario</t>
         </is>
       </c>
-      <c r="B159" s="14" t="inlineStr">
+      <c r="B159" s="15" t="inlineStr">
         <is>
           <t>Check the server rejects data requests without a signed-in session</t>
         </is>
       </c>
     </row>
     <row r="160" ht="15" customHeight="1">
-      <c r="A160" s="13" t="inlineStr">
+      <c r="A160" s="14" t="inlineStr">
         <is>
           <t>Pre-conditions</t>
         </is>
       </c>
-      <c r="B160" s="14" t="inlineStr">
+      <c r="B160" s="15" t="inlineStr">
         <is>
           <t>App running. User is signed out.</t>
         </is>
       </c>
     </row>
     <row r="161" ht="42" customHeight="1">
-      <c r="A161" s="13" t="inlineStr">
+      <c r="A161" s="14" t="inlineStr">
         <is>
           <t>Test Steps</t>
         </is>
       </c>
-      <c r="B161" s="14" t="inlineStr">
+      <c r="B161" s="15" t="inlineStr">
         <is>
           <t>1. Open http://localhost:3000/login
 2. Open DevTools (F12) &gt; Console and run:
@@ -2718,67 +2718,67 @@
       </c>
     </row>
     <row r="162" ht="15" customHeight="1">
-      <c r="A162" s="13" t="inlineStr">
+      <c r="A162" s="14" t="inlineStr">
         <is>
           <t>Test Data</t>
         </is>
       </c>
-      <c r="B162" s="14" t="inlineStr">
+      <c r="B162" s="15" t="inlineStr">
         <is>
           <t>No session</t>
         </is>
       </c>
     </row>
     <row r="163" ht="15" customHeight="1">
-      <c r="A163" s="13" t="inlineStr">
+      <c r="A163" s="14" t="inlineStr">
         <is>
           <t>Expected Result</t>
         </is>
       </c>
-      <c r="B163" s="14" t="inlineStr">
+      <c r="B163" s="15" t="inlineStr">
         <is>
           <t>Returns 401 ('Not signed in'); no venue data returned</t>
         </is>
       </c>
     </row>
     <row r="164" ht="15" customHeight="1">
-      <c r="A164" s="13" t="inlineStr">
+      <c r="A164" s="14" t="inlineStr">
         <is>
           <t>Created By</t>
         </is>
       </c>
-      <c r="B164" s="14" t="inlineStr">
+      <c r="B164" s="15" t="inlineStr">
         <is>
           <t>Zhenhan</t>
         </is>
       </c>
     </row>
     <row r="165" ht="15" customHeight="1">
-      <c r="A165" s="13" t="inlineStr">
+      <c r="A165" s="14" t="inlineStr">
         <is>
           <t>Date of Creation</t>
         </is>
       </c>
-      <c r="B165" s="14" t="inlineStr">
+      <c r="B165" s="15" t="inlineStr">
         <is>
           <t>06/10/2026</t>
         </is>
       </c>
     </row>
     <row r="166" ht="15" customHeight="1">
-      <c r="A166" s="15" t="inlineStr">
+      <c r="A166" s="16" t="inlineStr">
         <is>
           <t>Item</t>
         </is>
       </c>
-      <c r="B166" s="15" t="inlineStr">
+      <c r="B166" s="16" t="inlineStr">
         <is>
           <t>Details</t>
         </is>
       </c>
     </row>
     <row r="167" ht="15" customHeight="1">
-      <c r="A167" s="16" t="inlineStr">
+      <c r="A167" s="7" t="inlineStr">
         <is>
           <t>Actual Result</t>
         </is>
@@ -2790,7 +2790,7 @@
       </c>
     </row>
     <row r="168" ht="15" customHeight="1">
-      <c r="A168" s="16" t="inlineStr">
+      <c r="A168" s="7" t="inlineStr">
         <is>
           <t>Pass/Fail/Not Executed/Blocked</t>
         </is>
@@ -2802,7 +2802,7 @@
       </c>
     </row>
     <row r="169" ht="15" customHeight="1">
-      <c r="A169" s="16" t="inlineStr">
+      <c r="A169" s="7" t="inlineStr">
         <is>
           <t>Remarks</t>
         </is>
@@ -2814,7 +2814,7 @@
       </c>
     </row>
     <row r="170" ht="15" customHeight="1">
-      <c r="A170" s="16" t="inlineStr">
+      <c r="A170" s="7" t="inlineStr">
         <is>
           <t>Executed By</t>
         </is>
@@ -2826,7 +2826,7 @@
       </c>
     </row>
     <row r="171" ht="15" customHeight="1">
-      <c r="A171" s="16" t="inlineStr">
+      <c r="A171" s="7" t="inlineStr">
         <is>
           <t>Date of Execution</t>
         </is>
@@ -2838,48 +2838,48 @@
       </c>
     </row>
     <row r="174" ht="15" customHeight="1">
-      <c r="A174" s="12" t="inlineStr">
+      <c r="A174" s="13" t="inlineStr">
         <is>
           <t>Item</t>
         </is>
       </c>
-      <c r="B174" s="12" t="inlineStr">
+      <c r="B174" s="13" t="inlineStr">
         <is>
           <t>Details</t>
         </is>
       </c>
     </row>
     <row r="175" ht="15" customHeight="1">
-      <c r="A175" s="13" t="inlineStr">
+      <c r="A175" s="14" t="inlineStr">
         <is>
           <t>Test Case ID</t>
         </is>
       </c>
-      <c r="B175" s="14" t="inlineStr">
+      <c r="B175" s="15" t="inlineStr">
         <is>
           <t>TC-023</t>
         </is>
       </c>
     </row>
     <row r="176" ht="28" customHeight="1">
-      <c r="A176" s="13" t="inlineStr">
+      <c r="A176" s="14" t="inlineStr">
         <is>
           <t>Test Scenario</t>
         </is>
       </c>
-      <c r="B176" s="14" t="inlineStr">
+      <c r="B176" s="15" t="inlineStr">
         <is>
           <t>Check a user whose role is changed mid-session gets an authorisation error on their next action</t>
         </is>
       </c>
     </row>
     <row r="177" ht="42" customHeight="1">
-      <c r="A177" s="13" t="inlineStr">
+      <c r="A177" s="14" t="inlineStr">
         <is>
           <t>Pre-conditions</t>
         </is>
       </c>
-      <c r="B177" s="14" t="inlineStr">
+      <c r="B177" s="15" t="inlineStr">
         <is>
           <t>App running (frontend http://localhost:3000, backend on shared Supabase DB). Page freshly loaded (seed event data). Account active and not locked.
 Tester has Supabase dashboard access. AFTER TEST: set the role back to 'venue'.</t>
@@ -2887,12 +2887,12 @@
       </c>
     </row>
     <row r="178" ht="70" customHeight="1">
-      <c r="A178" s="13" t="inlineStr">
+      <c r="A178" s="14" t="inlineStr">
         <is>
           <t>Test Steps</t>
         </is>
       </c>
-      <c r="B178" s="14" t="inlineStr">
+      <c r="B178" s="15" t="inlineStr">
         <is>
           <t>1. Log in as venue staff and open Venue catalogue
 2. Click Edit on a venue (leave the form open)
@@ -2903,67 +2903,67 @@
       </c>
     </row>
     <row r="179" ht="15" customHeight="1">
-      <c r="A179" s="13" t="inlineStr">
+      <c r="A179" s="14" t="inlineStr">
         <is>
           <t>Test Data</t>
         </is>
       </c>
-      <c r="B179" s="14" t="inlineStr">
+      <c r="B179" s="15" t="inlineStr">
         <is>
           <t>Email=daniel.ortiz@connectsphere.edu; Password=&lt;team password&gt;</t>
         </is>
       </c>
     </row>
     <row r="180" ht="28" customHeight="1">
-      <c r="A180" s="13" t="inlineStr">
+      <c r="A180" s="14" t="inlineStr">
         <is>
           <t>Expected Result</t>
         </is>
       </c>
-      <c r="B180" s="14" t="inlineStr">
+      <c r="B180" s="15" t="inlineStr">
         <is>
           <t>Step 4: save is refused and an error 'You don't have permission to do that.' is shown; venue is unchanged</t>
         </is>
       </c>
     </row>
     <row r="181" ht="15" customHeight="1">
-      <c r="A181" s="13" t="inlineStr">
+      <c r="A181" s="14" t="inlineStr">
         <is>
           <t>Created By</t>
         </is>
       </c>
-      <c r="B181" s="14" t="inlineStr">
+      <c r="B181" s="15" t="inlineStr">
         <is>
           <t>Zhenhan</t>
         </is>
       </c>
     </row>
     <row r="182" ht="15" customHeight="1">
-      <c r="A182" s="13" t="inlineStr">
+      <c r="A182" s="14" t="inlineStr">
         <is>
           <t>Date of Creation</t>
         </is>
       </c>
-      <c r="B182" s="14" t="inlineStr">
+      <c r="B182" s="15" t="inlineStr">
         <is>
           <t>06/10/2026</t>
         </is>
       </c>
     </row>
     <row r="183" ht="15" customHeight="1">
-      <c r="A183" s="15" t="inlineStr">
+      <c r="A183" s="16" t="inlineStr">
         <is>
           <t>Item</t>
         </is>
       </c>
-      <c r="B183" s="15" t="inlineStr">
+      <c r="B183" s="16" t="inlineStr">
         <is>
           <t>Details</t>
         </is>
       </c>
     </row>
     <row r="184" ht="28" customHeight="1">
-      <c r="A184" s="16" t="inlineStr">
+      <c r="A184" s="7" t="inlineStr">
         <is>
           <t>Actual Result</t>
         </is>
@@ -2975,7 +2975,7 @@
       </c>
     </row>
     <row r="185" ht="15" customHeight="1">
-      <c r="A185" s="16" t="inlineStr">
+      <c r="A185" s="7" t="inlineStr">
         <is>
           <t>Pass/Fail/Not Executed/Blocked</t>
         </is>
@@ -2987,7 +2987,7 @@
       </c>
     </row>
     <row r="186" ht="15" customHeight="1">
-      <c r="A186" s="16" t="inlineStr">
+      <c r="A186" s="7" t="inlineStr">
         <is>
           <t>Remarks</t>
         </is>
@@ -2999,7 +2999,7 @@
       </c>
     </row>
     <row r="187" ht="15" customHeight="1">
-      <c r="A187" s="16" t="inlineStr">
+      <c r="A187" s="7" t="inlineStr">
         <is>
           <t>Executed By</t>
         </is>
@@ -3011,7 +3011,7 @@
       </c>
     </row>
     <row r="188" ht="15" customHeight="1">
-      <c r="A188" s="16" t="inlineStr">
+      <c r="A188" s="7" t="inlineStr">
         <is>
           <t>Date of Execution</t>
         </is>
@@ -3023,60 +3023,60 @@
       </c>
     </row>
     <row r="191" ht="15" customHeight="1">
-      <c r="A191" s="12" t="inlineStr">
+      <c r="A191" s="13" t="inlineStr">
         <is>
           <t>Item</t>
         </is>
       </c>
-      <c r="B191" s="12" t="inlineStr">
+      <c r="B191" s="13" t="inlineStr">
         <is>
           <t>Details</t>
         </is>
       </c>
     </row>
     <row r="192" ht="15" customHeight="1">
-      <c r="A192" s="13" t="inlineStr">
+      <c r="A192" s="14" t="inlineStr">
         <is>
           <t>Test Case ID</t>
         </is>
       </c>
-      <c r="B192" s="14" t="inlineStr">
+      <c r="B192" s="15" t="inlineStr">
         <is>
           <t>TC-024</t>
         </is>
       </c>
     </row>
     <row r="193" ht="15" customHeight="1">
-      <c r="A193" s="13" t="inlineStr">
+      <c r="A193" s="14" t="inlineStr">
         <is>
           <t>Test Scenario</t>
         </is>
       </c>
-      <c r="B193" s="14" t="inlineStr">
+      <c r="B193" s="15" t="inlineStr">
         <is>
           <t>Check event data and event actions are protected by the server, not only the interface</t>
         </is>
       </c>
     </row>
     <row r="194" ht="28" customHeight="1">
-      <c r="A194" s="13" t="inlineStr">
+      <c r="A194" s="14" t="inlineStr">
         <is>
           <t>Pre-conditions</t>
         </is>
       </c>
-      <c r="B194" s="14" t="inlineStr">
+      <c r="B194" s="15" t="inlineStr">
         <is>
           <t>App running (frontend http://localhost:3000, backend on shared Supabase DB). Page freshly loaded (seed event data). Account active and not locked.</t>
         </is>
       </c>
     </row>
     <row r="195" ht="70" customHeight="1">
-      <c r="A195" s="13" t="inlineStr">
+      <c r="A195" s="14" t="inlineStr">
         <is>
           <t>Test Steps</t>
         </is>
       </c>
-      <c r="B195" s="14" t="inlineStr">
+      <c r="B195" s="15" t="inlineStr">
         <is>
           <t>1. Log in as the attendee
 2. Open DevTools (F12) &gt; Console and run:
@@ -3086,67 +3086,67 @@
       </c>
     </row>
     <row r="196" ht="15" customHeight="1">
-      <c r="A196" s="13" t="inlineStr">
+      <c r="A196" s="14" t="inlineStr">
         <is>
           <t>Test Data</t>
         </is>
       </c>
-      <c r="B196" s="14" t="inlineStr">
+      <c r="B196" s="15" t="inlineStr">
         <is>
           <t>Email=sam.adeyemi@student.connectsphere.edu; Password=&lt;team password&gt;</t>
         </is>
       </c>
     </row>
     <row r="197" ht="42" customHeight="1">
-      <c r="A197" s="13" t="inlineStr">
+      <c r="A197" s="14" t="inlineStr">
         <is>
           <t>Expected Result</t>
         </is>
       </c>
-      <c r="B197" s="14" t="inlineStr">
+      <c r="B197" s="15" t="inlineStr">
         <is>
           <t>Event data is served by the backend only to authorised users: the attendee cannot obtain unpublished events (request is refused with 403, and 'Postgrad Mixer' is not present in data delivered to the browser)</t>
         </is>
       </c>
     </row>
     <row r="198" ht="15" customHeight="1">
-      <c r="A198" s="13" t="inlineStr">
+      <c r="A198" s="14" t="inlineStr">
         <is>
           <t>Created By</t>
         </is>
       </c>
-      <c r="B198" s="14" t="inlineStr">
+      <c r="B198" s="15" t="inlineStr">
         <is>
           <t>Zhenhan</t>
         </is>
       </c>
     </row>
     <row r="199" ht="15" customHeight="1">
-      <c r="A199" s="13" t="inlineStr">
+      <c r="A199" s="14" t="inlineStr">
         <is>
           <t>Date of Creation</t>
         </is>
       </c>
-      <c r="B199" s="14" t="inlineStr">
+      <c r="B199" s="15" t="inlineStr">
         <is>
           <t>06/10/2026</t>
         </is>
       </c>
     </row>
     <row r="200" ht="15" customHeight="1">
-      <c r="A200" s="15" t="inlineStr">
+      <c r="A200" s="16" t="inlineStr">
         <is>
           <t>Item</t>
         </is>
       </c>
-      <c r="B200" s="15" t="inlineStr">
+      <c r="B200" s="16" t="inlineStr">
         <is>
           <t>Details</t>
         </is>
       </c>
     </row>
     <row r="201" ht="42" customHeight="1">
-      <c r="A201" s="16" t="inlineStr">
+      <c r="A201" s="7" t="inlineStr">
         <is>
           <t>Actual Result</t>
         </is>
@@ -3158,19 +3158,19 @@
       </c>
     </row>
     <row r="202" ht="15" customHeight="1">
-      <c r="A202" s="16" t="inlineStr">
+      <c r="A202" s="7" t="inlineStr">
         <is>
           <t>Pass/Fail/Not Executed/Blocked</t>
         </is>
       </c>
-      <c r="B202" s="7" t="inlineStr">
+      <c r="B202" s="8" t="inlineStr">
         <is>
           <t>Blocked</t>
         </is>
       </c>
     </row>
     <row r="203" ht="15" customHeight="1">
-      <c r="A203" s="16" t="inlineStr">
+      <c r="A203" s="7" t="inlineStr">
         <is>
           <t>Remarks</t>
         </is>
@@ -3182,7 +3182,7 @@
       </c>
     </row>
     <row r="204" ht="15" customHeight="1">
-      <c r="A204" s="16" t="inlineStr">
+      <c r="A204" s="7" t="inlineStr">
         <is>
           <t>Executed By</t>
         </is>
@@ -3194,7 +3194,7 @@
       </c>
     </row>
     <row r="205" ht="15" customHeight="1">
-      <c r="A205" s="16" t="inlineStr">
+      <c r="A205" s="7" t="inlineStr">
         <is>
           <t>Date of Execution</t>
         </is>

</xml_diff>